<commit_message>
beaucoup de résultats grâce à excel
</commit_message>
<xml_diff>
--- a/excel/entree.xlsx
+++ b/excel/entree.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Feuille1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Feuille1!$A$1:$F$125</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Feuille1!$A$1:$F$115</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="11">
   <si>
     <t xml:space="preserve">nom</t>
   </si>
@@ -43,10 +43,19 @@
     <t xml:space="preserve">bruit</t>
   </si>
   <si>
-    <t xml:space="preserve">logo HX2</t>
+    <t xml:space="preserve">bounty</t>
   </si>
   <si>
     <t xml:space="preserve">mid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">classe HX2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">small</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HX2 tableau</t>
   </si>
 </sst>
 </file>
@@ -270,7 +279,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F115"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7.5"/>
@@ -309,16 +318,16 @@
         <v>7</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -329,16 +338,16 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -349,225 +358,537 @@
         <v>7</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E4" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="F12" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="F4" s="2" t="n">
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+      <c r="C13" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+      <c r="A14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
+      <c r="A15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+      <c r="A16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
+      <c r="A17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+      <c r="A18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
+      <c r="A19" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+      <c r="A20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
+      <c r="A21" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
+      <c r="A22" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
+      <c r="A23" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
+      <c r="A24" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
+      <c r="A25" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
+      <c r="A26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
+      <c r="A27" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
+      <c r="A28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
+      <c r="A29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
+      <c r="A30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="2"/>
@@ -612,49 +933,31 @@
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
       <c r="F36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
       <c r="F37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
       <c r="F38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
       <c r="F39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
       <c r="F40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
       <c r="F41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -692,31 +995,49 @@
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
       <c r="F46" s="2"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
       <c r="F47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
       <c r="F48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
       <c r="F49" s="2"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
       <c r="F50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
       <c r="F51" s="2"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -768,84 +1089,34 @@
       <c r="F57" s="2"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
-      <c r="F58" s="2"/>
+      <c r="A58" s="1"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-      <c r="E59" s="2"/>
-      <c r="F59" s="2"/>
+      <c r="A59" s="1"/>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="2"/>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
-      <c r="F60" s="2"/>
+      <c r="A60" s="1"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
-      <c r="F61" s="2"/>
+      <c r="A61" s="1"/>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
-      <c r="F62" s="2"/>
+      <c r="A62" s="1"/>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2"/>
-      <c r="C63" s="2"/>
-      <c r="D63" s="2"/>
-      <c r="E63" s="2"/>
-      <c r="F63" s="2"/>
+      <c r="A63" s="1"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="2"/>
-      <c r="B64" s="2"/>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
-      <c r="E64" s="2"/>
-      <c r="F64" s="2"/>
+      <c r="A64" s="1"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="2"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
-      <c r="F65" s="2"/>
+      <c r="A65" s="1"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
-      <c r="E66" s="2"/>
-      <c r="F66" s="2"/>
+      <c r="A66" s="1"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-      <c r="E67" s="2"/>
-      <c r="F67" s="2"/>
+      <c r="A67" s="1"/>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1"/>
@@ -991,38 +1262,8 @@
     <row r="115" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="1"/>
     </row>
-    <row r="116" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A116" s="1"/>
-    </row>
-    <row r="117" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A117" s="1"/>
-    </row>
-    <row r="118" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="1"/>
-    </row>
-    <row r="119" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A119" s="1"/>
-    </row>
-    <row r="120" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A120" s="1"/>
-    </row>
-    <row r="121" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A121" s="1"/>
-    </row>
-    <row r="122" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A122" s="1"/>
-    </row>
-    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A123" s="1"/>
-    </row>
-    <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A124" s="1"/>
-    </row>
-    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A125" s="1"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F125"/>
+  <autoFilter ref="A1:F115"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>